<commit_message>
40_line_build: short case (lap + RNPL cancellations on a budgeted cost base), with and without the Q4 marketing cut that holds the floor
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/ABNB_margin_line_build.xlsx
+++ b/model/ABNB_margin_line_build.xlsx
@@ -15,7 +15,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backcast" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vs_run23" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals_1Q23_2Q26" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Short_case" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Short_case_quarterly" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Short_case_revenue_path" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals_1Q23_2Q26" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,13 +493,1587 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>revenue_vs_team_path_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nights_yoy</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ops_cash</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ops_per_booking</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>chargebacks</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>interest_income</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sm_pct_rev</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>total_cash_costs_pct_rev</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>margin</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>margin_vs_base_pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3Q26</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4680.9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-2.563</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>374.971</v>
+      </c>
+      <c r="F2" t="n">
+        <v>9.442</v>
+      </c>
+      <c r="G2" t="n">
+        <v>34.551</v>
+      </c>
+      <c r="H2" t="n">
+        <v>174.359</v>
+      </c>
+      <c r="I2" t="n">
+        <v>16.627</v>
+      </c>
+      <c r="J2" t="n">
+        <v>51.523</v>
+      </c>
+      <c r="K2" t="n">
+        <v>48.918</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-1.449</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4Q26</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2965.868</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-6.678</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>329.176</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.387</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30.508</v>
+      </c>
+      <c r="H3" t="n">
+        <v>156.169</v>
+      </c>
+      <c r="I3" t="n">
+        <v>25.561</v>
+      </c>
+      <c r="J3" t="n">
+        <v>77.107</v>
+      </c>
+      <c r="K3" t="n">
+        <v>23.589</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-4.695</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1Q27</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2835.535</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-7.127</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>329.266</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7.297</v>
+      </c>
+      <c r="G4" t="n">
+        <v>39.258</v>
+      </c>
+      <c r="H4" t="n">
+        <v>167.126</v>
+      </c>
+      <c r="I4" t="n">
+        <v>29.246</v>
+      </c>
+      <c r="J4" t="n">
+        <v>88.004</v>
+      </c>
+      <c r="K4" t="n">
+        <v>12.724</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-5.488</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2Q27</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3762.972</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-6.602</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>352.014</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8.378</v>
+      </c>
+      <c r="G5" t="n">
+        <v>36.556</v>
+      </c>
+      <c r="H5" t="n">
+        <v>186.133</v>
+      </c>
+      <c r="I5" t="n">
+        <v>24.851</v>
+      </c>
+      <c r="J5" t="n">
+        <v>70.557</v>
+      </c>
+      <c r="K5" t="n">
+        <v>29.992</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-4.107</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3Q27</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4988.174</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-5.54</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>409.419</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9.872</v>
+      </c>
+      <c r="G6" t="n">
+        <v>36.082</v>
+      </c>
+      <c r="H6" t="n">
+        <v>176.877</v>
+      </c>
+      <c r="I6" t="n">
+        <v>16.437</v>
+      </c>
+      <c r="J6" t="n">
+        <v>51.317</v>
+      </c>
+      <c r="K6" t="n">
+        <v>49.097</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-2.866</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4Q27</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3326.831</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-4.009</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>360.088</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.738</v>
+      </c>
+      <c r="G7" t="n">
+        <v>32.169</v>
+      </c>
+      <c r="H7" t="n">
+        <v>160.888</v>
+      </c>
+      <c r="I7" t="n">
+        <v>26.31</v>
+      </c>
+      <c r="J7" t="n">
+        <v>75.881</v>
+      </c>
+      <c r="K7" t="n">
+        <v>24.739</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-3.257</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>revenue_musd</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gbv_busd</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nights_mm</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>nights_yoy_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>adr_reported_yoy_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>revenue_vs_base_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3Q26</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4680.9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.361</v>
+      </c>
+      <c r="D2" t="n">
+        <v>144.956</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-2.563</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4Q26</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2965.868</v>
+      </c>
+      <c r="C3" t="n">
+        <v>21.452</v>
+      </c>
+      <c r="D3" t="n">
+        <v>127.995</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-6.678</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1Q27</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2835.535</v>
+      </c>
+      <c r="C4" t="n">
+        <v>30.276</v>
+      </c>
+      <c r="D4" t="n">
+        <v>162.448</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.302</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-7.127</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2Q27</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3762.972</v>
+      </c>
+      <c r="C5" t="n">
+        <v>27.69</v>
+      </c>
+      <c r="D5" t="n">
+        <v>151.266</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.193</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-6.602</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3Q27</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4988.174</v>
+      </c>
+      <c r="C6" t="n">
+        <v>26.818</v>
+      </c>
+      <c r="D6" t="n">
+        <v>149.305</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-5.54</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4Q27</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3326.831</v>
+      </c>
+      <c r="C7" t="n">
+        <v>23.839</v>
+      </c>
+      <c r="D7" t="n">
+        <v>133.115</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.285</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-4.009</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nights_m</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>gbv_busd</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>cor_cash</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ops_cash</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>pd_cash</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>sm_cash</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ga_cash</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ga_cash_ex_lodging</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>lodging_tax_reserves</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>sbc_total_is</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>adj_ebitda_reported</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>adj_ebitda_margin_pct</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>interest_income</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>net_income</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>eps_diluted</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>shares_diluted_m</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>funds_held_on_behalf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1Q23</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1818</v>
+      </c>
+      <c r="C2" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>428</v>
+      </c>
+      <c r="F2" t="n">
+        <v>267</v>
+      </c>
+      <c r="G2" t="n">
+        <v>271</v>
+      </c>
+      <c r="H2" t="n">
+        <v>422</v>
+      </c>
+      <c r="I2" t="n">
+        <v>195</v>
+      </c>
+      <c r="J2" t="n">
+        <v>191</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>11</v>
+      </c>
+      <c r="M2" t="n">
+        <v>240</v>
+      </c>
+      <c r="N2" t="n">
+        <v>262</v>
+      </c>
+      <c r="O2" t="n">
+        <v>14.41</v>
+      </c>
+      <c r="P2" t="n">
+        <v>146</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>117</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="S2" t="n">
+        <v>670</v>
+      </c>
+      <c r="T2" t="n">
+        <v>7760</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2Q23</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2484</v>
+      </c>
+      <c r="C3" t="n">
+        <v>115.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>432</v>
+      </c>
+      <c r="F3" t="n">
+        <v>298</v>
+      </c>
+      <c r="G3" t="n">
+        <v>260</v>
+      </c>
+      <c r="H3" t="n">
+        <v>450</v>
+      </c>
+      <c r="I3" t="n">
+        <v>217</v>
+      </c>
+      <c r="J3" t="n">
+        <v>219</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L3" t="n">
+        <v>9</v>
+      </c>
+      <c r="M3" t="n">
+        <v>304</v>
+      </c>
+      <c r="N3" t="n">
+        <v>819</v>
+      </c>
+      <c r="O3" t="n">
+        <v>32.97</v>
+      </c>
+      <c r="P3" t="n">
+        <v>191</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>650</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="S3" t="n">
+        <v>665</v>
+      </c>
+      <c r="T3" t="n">
+        <v>9144</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3Q23</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3397</v>
+      </c>
+      <c r="C4" t="n">
+        <v>113.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>459</v>
+      </c>
+      <c r="F4" t="n">
+        <v>299</v>
+      </c>
+      <c r="G4" t="n">
+        <v>244</v>
+      </c>
+      <c r="H4" t="n">
+        <v>370</v>
+      </c>
+      <c r="I4" t="n">
+        <v>243</v>
+      </c>
+      <c r="J4" t="n">
+        <v>202</v>
+      </c>
+      <c r="K4" t="n">
+        <v>41</v>
+      </c>
+      <c r="L4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" t="n">
+        <v>286</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1834</v>
+      </c>
+      <c r="O4" t="n">
+        <v>53.99</v>
+      </c>
+      <c r="P4" t="n">
+        <v>192</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>4374</v>
+      </c>
+      <c r="R4" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="S4" t="n">
+        <v>660</v>
+      </c>
+      <c r="T4" t="n">
+        <v>5986</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4Q23</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2218</v>
+      </c>
+      <c r="C5" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>384</v>
+      </c>
+      <c r="F5" t="n">
+        <v>254</v>
+      </c>
+      <c r="G5" t="n">
+        <v>253</v>
+      </c>
+      <c r="H5" t="n">
+        <v>391</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1142</v>
+      </c>
+      <c r="J5" t="n">
+        <v>211</v>
+      </c>
+      <c r="K5" t="n">
+        <v>931</v>
+      </c>
+      <c r="L5" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" t="n">
+        <v>290</v>
+      </c>
+      <c r="N5" t="n">
+        <v>738</v>
+      </c>
+      <c r="O5" t="n">
+        <v>33.27</v>
+      </c>
+      <c r="P5" t="n">
+        <v>192</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-349</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="S5" t="n">
+        <v>640</v>
+      </c>
+      <c r="T5" t="n">
+        <v>5869</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1Q24</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2142</v>
+      </c>
+      <c r="C6" t="n">
+        <v>132.6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>480</v>
+      </c>
+      <c r="F6" t="n">
+        <v>266</v>
+      </c>
+      <c r="G6" t="n">
+        <v>290</v>
+      </c>
+      <c r="H6" t="n">
+        <v>479</v>
+      </c>
+      <c r="I6" t="n">
+        <v>231</v>
+      </c>
+      <c r="J6" t="n">
+        <v>223</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M6" t="n">
+        <v>295</v>
+      </c>
+      <c r="N6" t="n">
+        <v>424</v>
+      </c>
+      <c r="O6" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="P6" t="n">
+        <v>202</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>264</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="S6" t="n">
+        <v>654</v>
+      </c>
+      <c r="T6" t="n">
+        <v>8737</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2Q24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2748</v>
+      </c>
+      <c r="C7" t="n">
+        <v>125.1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>506</v>
+      </c>
+      <c r="F7" t="n">
+        <v>314</v>
+      </c>
+      <c r="G7" t="n">
+        <v>280</v>
+      </c>
+      <c r="H7" t="n">
+        <v>527</v>
+      </c>
+      <c r="I7" t="n">
+        <v>242</v>
+      </c>
+      <c r="J7" t="n">
+        <v>242</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>14</v>
+      </c>
+      <c r="M7" t="n">
+        <v>382</v>
+      </c>
+      <c r="N7" t="n">
+        <v>894</v>
+      </c>
+      <c r="O7" t="n">
+        <v>32.53</v>
+      </c>
+      <c r="P7" t="n">
+        <v>226</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>555</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="S7" t="n">
+        <v>649</v>
+      </c>
+      <c r="T7" t="n">
+        <v>10342</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3Q24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3732</v>
+      </c>
+      <c r="C8" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>465</v>
+      </c>
+      <c r="F8" t="n">
+        <v>347</v>
+      </c>
+      <c r="G8" t="n">
+        <v>294</v>
+      </c>
+      <c r="H8" t="n">
+        <v>471</v>
+      </c>
+      <c r="I8" t="n">
+        <v>268</v>
+      </c>
+      <c r="J8" t="n">
+        <v>210</v>
+      </c>
+      <c r="K8" t="n">
+        <v>58</v>
+      </c>
+      <c r="L8" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" t="n">
+        <v>362</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1958</v>
+      </c>
+      <c r="O8" t="n">
+        <v>52.47</v>
+      </c>
+      <c r="P8" t="n">
+        <v>207</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1368</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="S8" t="n">
+        <v>642</v>
+      </c>
+      <c r="T8" t="n">
+        <v>6573</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4Q24</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2480</v>
+      </c>
+      <c r="C9" t="n">
+        <v>111</v>
+      </c>
+      <c r="D9" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>427</v>
+      </c>
+      <c r="F9" t="n">
+        <v>265</v>
+      </c>
+      <c r="G9" t="n">
+        <v>306</v>
+      </c>
+      <c r="H9" t="n">
+        <v>501</v>
+      </c>
+      <c r="I9" t="n">
+        <v>183</v>
+      </c>
+      <c r="J9" t="n">
+        <v>226</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-43</v>
+      </c>
+      <c r="L9" t="n">
+        <v>22</v>
+      </c>
+      <c r="M9" t="n">
+        <v>368</v>
+      </c>
+      <c r="N9" t="n">
+        <v>765</v>
+      </c>
+      <c r="O9" t="n">
+        <v>30.85</v>
+      </c>
+      <c r="P9" t="n">
+        <v>183</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>461</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="S9" t="n">
+        <v>636</v>
+      </c>
+      <c r="T9" t="n">
+        <v>5931</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1Q25</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2272</v>
+      </c>
+      <c r="C10" t="n">
+        <v>143.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>506</v>
+      </c>
+      <c r="F10" t="n">
+        <v>282</v>
+      </c>
+      <c r="G10" t="n">
+        <v>338</v>
+      </c>
+      <c r="H10" t="n">
+        <v>519</v>
+      </c>
+      <c r="I10" t="n">
+        <v>231</v>
+      </c>
+      <c r="J10" t="n">
+        <v>235</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-4</v>
+      </c>
+      <c r="L10" t="n">
+        <v>25</v>
+      </c>
+      <c r="M10" t="n">
+        <v>358</v>
+      </c>
+      <c r="N10" t="n">
+        <v>417</v>
+      </c>
+      <c r="O10" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="P10" t="n">
+        <v>173</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>154</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="S10" t="n">
+        <v>632</v>
+      </c>
+      <c r="T10" t="n">
+        <v>9175</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2Q25</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3096</v>
+      </c>
+      <c r="C11" t="n">
+        <v>134.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>544</v>
+      </c>
+      <c r="F11" t="n">
+        <v>309</v>
+      </c>
+      <c r="G11" t="n">
+        <v>331</v>
+      </c>
+      <c r="H11" t="n">
+        <v>639</v>
+      </c>
+      <c r="I11" t="n">
+        <v>237</v>
+      </c>
+      <c r="J11" t="n">
+        <v>244</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-7</v>
+      </c>
+      <c r="L11" t="n">
+        <v>21</v>
+      </c>
+      <c r="M11" t="n">
+        <v>424</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1043</v>
+      </c>
+      <c r="O11" t="n">
+        <v>33.69</v>
+      </c>
+      <c r="P11" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>642</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="S11" t="n">
+        <v>626</v>
+      </c>
+      <c r="T11" t="n">
+        <v>11067</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3Q25</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4095</v>
+      </c>
+      <c r="C12" t="n">
+        <v>133.6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="E12" t="n">
+        <v>549</v>
+      </c>
+      <c r="F12" t="n">
+        <v>343</v>
+      </c>
+      <c r="G12" t="n">
+        <v>333</v>
+      </c>
+      <c r="H12" t="n">
+        <v>585</v>
+      </c>
+      <c r="I12" t="n">
+        <v>261</v>
+      </c>
+      <c r="J12" t="n">
+        <v>257</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4</v>
+      </c>
+      <c r="L12" t="n">
+        <v>22</v>
+      </c>
+      <c r="M12" t="n">
+        <v>399</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2051</v>
+      </c>
+      <c r="O12" t="n">
+        <v>50.09</v>
+      </c>
+      <c r="P12" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1374</v>
+      </c>
+      <c r="R12" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="S12" t="n">
+        <v>621</v>
+      </c>
+      <c r="T12" t="n">
+        <v>7209</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>4Q25</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2778</v>
+      </c>
+      <c r="C13" t="n">
+        <v>121.9</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>487</v>
+      </c>
+      <c r="F13" t="n">
+        <v>303</v>
+      </c>
+      <c r="G13" t="n">
+        <v>335</v>
+      </c>
+      <c r="H13" t="n">
+        <v>633</v>
+      </c>
+      <c r="I13" t="n">
+        <v>340</v>
+      </c>
+      <c r="J13" t="n">
+        <v>259</v>
+      </c>
+      <c r="K13" t="n">
+        <v>81</v>
+      </c>
+      <c r="L13" t="n">
+        <v>23</v>
+      </c>
+      <c r="M13" t="n">
+        <v>411</v>
+      </c>
+      <c r="N13" t="n">
+        <v>786</v>
+      </c>
+      <c r="O13" t="n">
+        <v>28.29</v>
+      </c>
+      <c r="P13" t="n">
+        <v>162</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>341</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="S13" t="n">
+        <v>614</v>
+      </c>
+      <c r="T13" t="n">
+        <v>6959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1Q26</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2678</v>
+      </c>
+      <c r="C14" t="n">
+        <v>156.2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>581</v>
+      </c>
+      <c r="F14" t="n">
+        <v>301</v>
+      </c>
+      <c r="G14" t="n">
+        <v>375</v>
+      </c>
+      <c r="H14" t="n">
+        <v>696</v>
+      </c>
+      <c r="I14" t="n">
+        <v>229</v>
+      </c>
+      <c r="J14" t="n">
+        <v>226</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>22</v>
+      </c>
+      <c r="M14" t="n">
+        <v>410</v>
+      </c>
+      <c r="N14" t="n">
+        <v>519</v>
+      </c>
+      <c r="O14" t="n">
+        <v>19.38</v>
+      </c>
+      <c r="P14" t="n">
+        <v>155</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>160</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="S14" t="n">
+        <v>608</v>
+      </c>
+      <c r="T14" t="n">
+        <v>10550</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2Q26</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3608</v>
+      </c>
+      <c r="C15" t="n">
+        <v>148.3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>633</v>
+      </c>
+      <c r="F15" t="n">
+        <v>323</v>
+      </c>
+      <c r="G15" t="n">
+        <v>374</v>
+      </c>
+      <c r="H15" t="n">
+        <v>808</v>
+      </c>
+      <c r="I15" t="n">
+        <v>225</v>
+      </c>
+      <c r="J15" t="n">
+        <v>227</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>17</v>
+      </c>
+      <c r="M15" t="n">
+        <v>487</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1261</v>
+      </c>
+      <c r="O15" t="n">
+        <v>34.95</v>
+      </c>
+      <c r="P15" t="n">
+        <v>183</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>816</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="S15" t="n">
+        <v>597</v>
+      </c>
+      <c r="T15" t="n">
+        <v>12224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1509,93 +3086,93 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>below</t>
+          <t>overlay</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>da_per_q</t>
+          <t>rnpl_ops_uplift_pct</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>20.63397059990752</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>20.63397059990752</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>20.63397059990752</v>
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>USD m per quarter</t>
+          <t>% uplift on ops &amp; support per completed booking</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>M7 parameter sheet</t>
+          <t>Cancellations raise contacts, refunds and make-goods per completed stay: 2Q26 10-Q customer relations +$10M on higher make-good payouts and related case reserves, 1Q26 +$3M refunds and credits; short case 4%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>below</t>
+          <t>overlay</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>sbc_growth</t>
+          <t>chargeback_add_per_booking</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>13.17774076718567</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>13.17774076718567</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>13.17774076718567</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>% y/y on SBC[q-4]</t>
+          <t>USD per booking added</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>M7 (recency-weighted last-4 y/y); mgmt: SBC growth below FY25's</t>
+          <t>1H26 chargebacks +$25M y/y (+37%) after two years of declines; short case +$0.15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>below</t>
+          <t>overlay</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>interest_income_beta</t>
+          <t>q4_marketing_cut_musd</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.8764975067193741</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>0.8764975067193741</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>0.8764975067193741</v>
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>x 3m T-bill x avg earning base / 4</t>
+          <t>USD m cut from 4Q26 marketing</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>M7 / WS04 rule (r 0.83, n 18)</t>
+          <t>Management protected the FY floor in 4Q24 by phasing brand marketing down; the short case reports the cut needed</t>
         </is>
       </c>
     </row>
@@ -1607,26 +3184,26 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tbill_3m</t>
+          <t>da_per_q</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3.76</v>
+        <v>20.63397059990752</v>
       </c>
       <c r="D36" t="n">
-        <v>3.76</v>
+        <v>20.63397059990752</v>
       </c>
       <c r="E36" t="n">
-        <v>3.76</v>
+        <v>20.63397059990752</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>% (3Q26 QTD average, held)</t>
+          <t>USD m per quarter</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>FRED DTB3 via M7</t>
+          <t>M7 parameter sheet</t>
         </is>
       </c>
     </row>
@@ -1638,26 +3215,26 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>cash_plus_sti</t>
+          <t>sbc_growth</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>12069</v>
+        <v>13.17774076718567</v>
       </c>
       <c r="D37" t="n">
-        <v>12069</v>
+        <v>13.17774076718567</v>
       </c>
       <c r="E37" t="n">
-        <v>12069</v>
+        <v>13.17774076718567</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>USD m, held flat</t>
+          <t>% y/y on SBC[q-4]</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>WS02 2Q26</t>
+          <t>M7 (recency-weighted last-4 y/y); mgmt: SBC growth below FY25's</t>
         </is>
       </c>
     </row>
@@ -1669,26 +3246,26 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>rnpl_share_shift_pts</t>
+          <t>interest_income_beta</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.8764975067193741</v>
       </c>
       <c r="D38" t="n">
-        <v>10</v>
+        <v>0.8764975067193741</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>0.8764975067193741</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>pts of GBV paid at check-in rather than at booking, vs 2025</t>
+          <t>x 3m T-bill x avg earning base / 4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No RNPL share series exists in the repo; sensitivity only: each 10 pts of GBV paid later cuts average funds held by ~10%</t>
+          <t>M7 / WS04 rule (r 0.83, n 18)</t>
         </is>
       </c>
     </row>
@@ -1700,26 +3277,26 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>interest_expense_per_q</t>
+          <t>tbill_3m</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>37</v>
+        <v>3.76</v>
       </c>
       <c r="D39" t="n">
-        <v>37</v>
+        <v>3.76</v>
       </c>
       <c r="E39" t="n">
-        <v>37</v>
+        <v>3.76</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>USD m per quarter</t>
+          <t>% (3Q26 QTD average, held)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>M7: $2.5bn notes (~$119M a year, WS05 H10)</t>
+          <t>FRED DTB3 via M7</t>
         </is>
       </c>
     </row>
@@ -1731,26 +3308,26 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>other_income_per_q</t>
+          <t>cash_plus_sti</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3.7</v>
+        <v>12069</v>
       </c>
       <c r="D40" t="n">
-        <v>3.7</v>
+        <v>12069</v>
       </c>
       <c r="E40" t="n">
-        <v>3.7</v>
+        <v>12069</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>USD m per quarter</t>
+          <t>USD m, held flat</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>M7 recency-weighted mean</t>
+          <t>WS02 2Q26</t>
         </is>
       </c>
     </row>
@@ -1762,26 +3339,26 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>etr_2h26</t>
+          <t>rnpl_share_shift_pts</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E41" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>% applied to 2H26 forecast quarters (1H26 printed 17.1%)</t>
+          <t>pts of GBV paid at check-in rather than at booking, vs 2025</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>M7; mgmt high teens (2Q26)</t>
+          <t>No RNPL share series exists in the repo; sensitivity only: each 10 pts of GBV paid later cuts average funds held by ~10%</t>
         </is>
       </c>
     </row>
@@ -1793,26 +3370,26 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>etr_fy27</t>
+          <t>interest_expense_per_q</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>17.5</v>
+        <v>37</v>
       </c>
       <c r="D42" t="n">
-        <v>17.5</v>
+        <v>37</v>
       </c>
       <c r="E42" t="n">
-        <v>17.5</v>
+        <v>37</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD m per quarter</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>M7; long-term mid-to-high teens under OBBBA (WS05 H09)</t>
+          <t>M7: $2.5bn notes (~$119M a year, WS05 H10)</t>
         </is>
       </c>
     </row>
@@ -1824,26 +3401,26 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>diluted_shares_2q26</t>
+          <t>other_income_per_q</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>597</v>
+        <v>3.7</v>
       </c>
       <c r="D43" t="n">
-        <v>597</v>
+        <v>3.7</v>
       </c>
       <c r="E43" t="n">
-        <v>597</v>
+        <v>3.7</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>USD m per quarter</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>WS02 2Q26</t>
+          <t>M7 recency-weighted mean</t>
         </is>
       </c>
     </row>
@@ -1855,24 +3432,117 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>etr_2h26</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>18</v>
+      </c>
+      <c r="D44" t="n">
+        <v>18</v>
+      </c>
+      <c r="E44" t="n">
+        <v>18</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>% applied to 2H26 forecast quarters (1H26 printed 17.1%)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>M7; mgmt high teens (2Q26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>below</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>etr_fy27</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E45" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>M7; long-term mid-to-high teens under OBBBA (WS05 H09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>below</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>diluted_shares_2q26</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>597</v>
+      </c>
+      <c r="D46" t="n">
+        <v>597</v>
+      </c>
+      <c r="E46" t="n">
+        <v>597</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>WS02 2Q26</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>below</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>diluted_shares_delta_per_q</t>
         </is>
       </c>
-      <c r="C44" t="n">
+      <c r="C47" t="n">
         <v>-5.324186618094461</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D47" t="n">
         <v>-5.324186618094461</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E47" t="n">
         <v>-5.324186618094461</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>m per quarter</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>M7: -buyback/price + issuance; authorisation runs out ~1Q27 (WS05 H11)</t>
         </is>
@@ -14805,10 +16475,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -14824,1008 +16494,192 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>quarter</t>
+          <t>case</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>q3_ebitda</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>nights_m</t>
+          <t>q3_margin</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>gbv_busd</t>
+          <t>q3_revenue</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>cor_cash</t>
+          <t>q4_ebitda</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ops_cash</t>
+          <t>q4_margin</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>pd_cash</t>
+          <t>q4_revenue</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>sm_cash</t>
+          <t>fy26_ebitda</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ga_cash</t>
+          <t>fy26_margin</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ga_cash_ex_lodging</t>
+          <t>fy26_revenue</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>lodging_tax_reserves</t>
+          <t>fy27_ebitda</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>fy27_margin</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>sbc_total_is</t>
+          <t>fy27_revenue</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>adj_ebitda_reported</t>
+          <t>q3_eps</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>adj_ebitda_margin_pct</t>
+          <t>fy27_eps</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>interest_income</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>net_income</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>eps_diluted</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>shares_diluted_m</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>funds_held_on_behalf</t>
+          <t>q4_marketing_cut_musd</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1Q23</t>
+          <t>short_costs_at_budget</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1818</v>
+        <v>2289.815</v>
       </c>
       <c r="C2" t="n">
-        <v>121.1</v>
+        <v>48.918</v>
       </c>
       <c r="D2" t="n">
-        <v>20.4</v>
+        <v>4680.9</v>
       </c>
       <c r="E2" t="n">
-        <v>428</v>
+        <v>699.6079999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>267</v>
+        <v>23.589</v>
       </c>
       <c r="G2" t="n">
-        <v>271</v>
+        <v>2965.868</v>
       </c>
       <c r="H2" t="n">
-        <v>422</v>
+        <v>4769.423</v>
       </c>
       <c r="I2" t="n">
-        <v>195</v>
+        <v>34.232</v>
       </c>
       <c r="J2" t="n">
-        <v>191</v>
+        <v>13932.768</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>4761.435</v>
       </c>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>31.927</v>
       </c>
       <c r="M2" t="n">
-        <v>240</v>
+        <v>14913.512</v>
       </c>
       <c r="N2" t="n">
-        <v>262</v>
+        <v>2.714</v>
       </c>
       <c r="O2" t="n">
-        <v>14.41</v>
+        <v>4.584</v>
       </c>
       <c r="P2" t="n">
-        <v>146</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>117</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S2" t="n">
-        <v>670</v>
-      </c>
-      <c r="T2" t="n">
-        <v>7760</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2Q23</t>
+          <t>short_with_q4_marketing_cut</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2484</v>
+        <v>2289.815</v>
       </c>
       <c r="C3" t="n">
-        <v>115.1</v>
+        <v>48.918</v>
       </c>
       <c r="D3" t="n">
-        <v>19.1</v>
+        <v>4680.9</v>
       </c>
       <c r="E3" t="n">
-        <v>432</v>
+        <v>876.317</v>
       </c>
       <c r="F3" t="n">
-        <v>298</v>
+        <v>29.547</v>
       </c>
       <c r="G3" t="n">
-        <v>260</v>
+        <v>2965.868</v>
       </c>
       <c r="H3" t="n">
-        <v>450</v>
+        <v>4946.133</v>
       </c>
       <c r="I3" t="n">
-        <v>217</v>
+        <v>35.5</v>
       </c>
       <c r="J3" t="n">
-        <v>219</v>
+        <v>13932.768</v>
       </c>
       <c r="K3" t="n">
-        <v>-2</v>
+        <v>4761.435</v>
       </c>
       <c r="L3" t="n">
-        <v>9</v>
+        <v>31.927</v>
       </c>
       <c r="M3" t="n">
-        <v>304</v>
+        <v>14913.512</v>
       </c>
       <c r="N3" t="n">
-        <v>819</v>
+        <v>2.714</v>
       </c>
       <c r="O3" t="n">
-        <v>32.97</v>
+        <v>4.584</v>
       </c>
       <c r="P3" t="n">
-        <v>191</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>650</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="S3" t="n">
-        <v>665</v>
-      </c>
-      <c r="T3" t="n">
-        <v>9144</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3Q23</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3397</v>
-      </c>
-      <c r="C4" t="n">
-        <v>113.2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>459</v>
-      </c>
-      <c r="F4" t="n">
-        <v>299</v>
-      </c>
-      <c r="G4" t="n">
-        <v>244</v>
-      </c>
-      <c r="H4" t="n">
-        <v>370</v>
-      </c>
-      <c r="I4" t="n">
-        <v>243</v>
-      </c>
-      <c r="J4" t="n">
-        <v>202</v>
-      </c>
-      <c r="K4" t="n">
-        <v>41</v>
-      </c>
-      <c r="L4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M4" t="n">
-        <v>286</v>
-      </c>
-      <c r="N4" t="n">
-        <v>1834</v>
-      </c>
-      <c r="O4" t="n">
-        <v>53.99</v>
-      </c>
-      <c r="P4" t="n">
-        <v>192</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>4374</v>
-      </c>
-      <c r="R4" t="n">
-        <v>6.63</v>
-      </c>
-      <c r="S4" t="n">
-        <v>660</v>
-      </c>
-      <c r="T4" t="n">
-        <v>5986</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4Q23</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2218</v>
-      </c>
-      <c r="C5" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="D5" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>384</v>
-      </c>
-      <c r="F5" t="n">
-        <v>254</v>
-      </c>
-      <c r="G5" t="n">
-        <v>253</v>
-      </c>
-      <c r="H5" t="n">
-        <v>391</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1142</v>
-      </c>
-      <c r="J5" t="n">
-        <v>211</v>
-      </c>
-      <c r="K5" t="n">
-        <v>931</v>
-      </c>
-      <c r="L5" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" t="n">
-        <v>290</v>
-      </c>
-      <c r="N5" t="n">
-        <v>738</v>
-      </c>
-      <c r="O5" t="n">
-        <v>33.27</v>
-      </c>
-      <c r="P5" t="n">
-        <v>192</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>-349</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-0.55</v>
-      </c>
-      <c r="S5" t="n">
-        <v>640</v>
-      </c>
-      <c r="T5" t="n">
-        <v>5869</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1Q24</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2142</v>
-      </c>
-      <c r="C6" t="n">
-        <v>132.6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="E6" t="n">
-        <v>480</v>
-      </c>
-      <c r="F6" t="n">
-        <v>266</v>
-      </c>
-      <c r="G6" t="n">
-        <v>290</v>
-      </c>
-      <c r="H6" t="n">
-        <v>479</v>
-      </c>
-      <c r="I6" t="n">
-        <v>231</v>
-      </c>
-      <c r="J6" t="n">
-        <v>223</v>
-      </c>
-      <c r="K6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" t="n">
-        <v>14</v>
-      </c>
-      <c r="M6" t="n">
-        <v>295</v>
-      </c>
-      <c r="N6" t="n">
-        <v>424</v>
-      </c>
-      <c r="O6" t="n">
-        <v>19.79</v>
-      </c>
-      <c r="P6" t="n">
-        <v>202</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>264</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="S6" t="n">
-        <v>654</v>
-      </c>
-      <c r="T6" t="n">
-        <v>8737</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2Q24</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2748</v>
-      </c>
-      <c r="C7" t="n">
-        <v>125.1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="E7" t="n">
-        <v>506</v>
-      </c>
-      <c r="F7" t="n">
-        <v>314</v>
-      </c>
-      <c r="G7" t="n">
-        <v>280</v>
-      </c>
-      <c r="H7" t="n">
-        <v>527</v>
-      </c>
-      <c r="I7" t="n">
-        <v>242</v>
-      </c>
-      <c r="J7" t="n">
-        <v>242</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>14</v>
-      </c>
-      <c r="M7" t="n">
-        <v>382</v>
-      </c>
-      <c r="N7" t="n">
-        <v>894</v>
-      </c>
-      <c r="O7" t="n">
-        <v>32.53</v>
-      </c>
-      <c r="P7" t="n">
-        <v>226</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>555</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="S7" t="n">
-        <v>649</v>
-      </c>
-      <c r="T7" t="n">
-        <v>10342</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3Q24</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3732</v>
-      </c>
-      <c r="C8" t="n">
-        <v>122.8</v>
-      </c>
-      <c r="D8" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>465</v>
-      </c>
-      <c r="F8" t="n">
-        <v>347</v>
-      </c>
-      <c r="G8" t="n">
-        <v>294</v>
-      </c>
-      <c r="H8" t="n">
-        <v>471</v>
-      </c>
-      <c r="I8" t="n">
-        <v>268</v>
-      </c>
-      <c r="J8" t="n">
-        <v>210</v>
-      </c>
-      <c r="K8" t="n">
-        <v>58</v>
-      </c>
-      <c r="L8" t="n">
-        <v>15</v>
-      </c>
-      <c r="M8" t="n">
-        <v>362</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1958</v>
-      </c>
-      <c r="O8" t="n">
-        <v>52.47</v>
-      </c>
-      <c r="P8" t="n">
-        <v>207</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>1368</v>
-      </c>
-      <c r="R8" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="S8" t="n">
-        <v>642</v>
-      </c>
-      <c r="T8" t="n">
-        <v>6573</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>4Q24</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2480</v>
-      </c>
-      <c r="C9" t="n">
-        <v>111</v>
-      </c>
-      <c r="D9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="E9" t="n">
-        <v>427</v>
-      </c>
-      <c r="F9" t="n">
-        <v>265</v>
-      </c>
-      <c r="G9" t="n">
-        <v>306</v>
-      </c>
-      <c r="H9" t="n">
-        <v>501</v>
-      </c>
-      <c r="I9" t="n">
-        <v>183</v>
-      </c>
-      <c r="J9" t="n">
-        <v>226</v>
-      </c>
-      <c r="K9" t="n">
-        <v>-43</v>
-      </c>
-      <c r="L9" t="n">
-        <v>22</v>
-      </c>
-      <c r="M9" t="n">
-        <v>368</v>
-      </c>
-      <c r="N9" t="n">
-        <v>765</v>
-      </c>
-      <c r="O9" t="n">
-        <v>30.85</v>
-      </c>
-      <c r="P9" t="n">
-        <v>183</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>461</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="S9" t="n">
-        <v>636</v>
-      </c>
-      <c r="T9" t="n">
-        <v>5931</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1Q25</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2272</v>
-      </c>
-      <c r="C10" t="n">
-        <v>143.1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>506</v>
-      </c>
-      <c r="F10" t="n">
-        <v>282</v>
-      </c>
-      <c r="G10" t="n">
-        <v>338</v>
-      </c>
-      <c r="H10" t="n">
-        <v>519</v>
-      </c>
-      <c r="I10" t="n">
-        <v>231</v>
-      </c>
-      <c r="J10" t="n">
-        <v>235</v>
-      </c>
-      <c r="K10" t="n">
-        <v>-4</v>
-      </c>
-      <c r="L10" t="n">
-        <v>25</v>
-      </c>
-      <c r="M10" t="n">
-        <v>358</v>
-      </c>
-      <c r="N10" t="n">
-        <v>417</v>
-      </c>
-      <c r="O10" t="n">
-        <v>18.35</v>
-      </c>
-      <c r="P10" t="n">
-        <v>173</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>154</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="S10" t="n">
-        <v>632</v>
-      </c>
-      <c r="T10" t="n">
-        <v>9175</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2Q25</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3096</v>
-      </c>
-      <c r="C11" t="n">
-        <v>134.4</v>
-      </c>
-      <c r="D11" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>544</v>
-      </c>
-      <c r="F11" t="n">
-        <v>309</v>
-      </c>
-      <c r="G11" t="n">
-        <v>331</v>
-      </c>
-      <c r="H11" t="n">
-        <v>639</v>
-      </c>
-      <c r="I11" t="n">
-        <v>237</v>
-      </c>
-      <c r="J11" t="n">
-        <v>244</v>
-      </c>
-      <c r="K11" t="n">
-        <v>-7</v>
-      </c>
-      <c r="L11" t="n">
-        <v>21</v>
-      </c>
-      <c r="M11" t="n">
-        <v>424</v>
-      </c>
-      <c r="N11" t="n">
-        <v>1043</v>
-      </c>
-      <c r="O11" t="n">
-        <v>33.69</v>
-      </c>
-      <c r="P11" t="n">
-        <v>190</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>642</v>
-      </c>
-      <c r="R11" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="S11" t="n">
-        <v>626</v>
-      </c>
-      <c r="T11" t="n">
-        <v>11067</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>3Q25</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>4095</v>
-      </c>
-      <c r="C12" t="n">
-        <v>133.6</v>
-      </c>
-      <c r="D12" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="E12" t="n">
-        <v>549</v>
-      </c>
-      <c r="F12" t="n">
-        <v>343</v>
-      </c>
-      <c r="G12" t="n">
-        <v>333</v>
-      </c>
-      <c r="H12" t="n">
-        <v>585</v>
-      </c>
-      <c r="I12" t="n">
-        <v>261</v>
-      </c>
-      <c r="J12" t="n">
-        <v>257</v>
-      </c>
-      <c r="K12" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" t="n">
-        <v>22</v>
-      </c>
-      <c r="M12" t="n">
-        <v>399</v>
-      </c>
-      <c r="N12" t="n">
-        <v>2051</v>
-      </c>
-      <c r="O12" t="n">
-        <v>50.09</v>
-      </c>
-      <c r="P12" t="n">
-        <v>180</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>1374</v>
-      </c>
-      <c r="R12" t="n">
-        <v>2.21</v>
-      </c>
-      <c r="S12" t="n">
-        <v>621</v>
-      </c>
-      <c r="T12" t="n">
-        <v>7209</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>4Q25</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>2778</v>
-      </c>
-      <c r="C13" t="n">
-        <v>121.9</v>
-      </c>
-      <c r="D13" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="E13" t="n">
-        <v>487</v>
-      </c>
-      <c r="F13" t="n">
-        <v>303</v>
-      </c>
-      <c r="G13" t="n">
-        <v>335</v>
-      </c>
-      <c r="H13" t="n">
-        <v>633</v>
-      </c>
-      <c r="I13" t="n">
-        <v>340</v>
-      </c>
-      <c r="J13" t="n">
-        <v>259</v>
-      </c>
-      <c r="K13" t="n">
-        <v>81</v>
-      </c>
-      <c r="L13" t="n">
-        <v>23</v>
-      </c>
-      <c r="M13" t="n">
-        <v>411</v>
-      </c>
-      <c r="N13" t="n">
-        <v>786</v>
-      </c>
-      <c r="O13" t="n">
-        <v>28.29</v>
-      </c>
-      <c r="P13" t="n">
-        <v>162</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>341</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="S13" t="n">
-        <v>614</v>
-      </c>
-      <c r="T13" t="n">
-        <v>6959</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1Q26</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2678</v>
-      </c>
-      <c r="C14" t="n">
-        <v>156.2</v>
-      </c>
-      <c r="D14" t="n">
-        <v>29.2</v>
-      </c>
-      <c r="E14" t="n">
-        <v>581</v>
-      </c>
-      <c r="F14" t="n">
-        <v>301</v>
-      </c>
-      <c r="G14" t="n">
-        <v>375</v>
-      </c>
-      <c r="H14" t="n">
-        <v>696</v>
-      </c>
-      <c r="I14" t="n">
-        <v>229</v>
-      </c>
-      <c r="J14" t="n">
-        <v>226</v>
-      </c>
-      <c r="K14" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" t="n">
-        <v>22</v>
-      </c>
-      <c r="M14" t="n">
-        <v>410</v>
-      </c>
-      <c r="N14" t="n">
-        <v>519</v>
-      </c>
-      <c r="O14" t="n">
-        <v>19.38</v>
-      </c>
-      <c r="P14" t="n">
-        <v>155</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>160</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="S14" t="n">
-        <v>608</v>
-      </c>
-      <c r="T14" t="n">
-        <v>10550</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2Q26</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3608</v>
-      </c>
-      <c r="C15" t="n">
-        <v>148.3</v>
-      </c>
-      <c r="D15" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="E15" t="n">
-        <v>633</v>
-      </c>
-      <c r="F15" t="n">
-        <v>323</v>
-      </c>
-      <c r="G15" t="n">
-        <v>374</v>
-      </c>
-      <c r="H15" t="n">
-        <v>808</v>
-      </c>
-      <c r="I15" t="n">
-        <v>225</v>
-      </c>
-      <c r="J15" t="n">
-        <v>227</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>17</v>
-      </c>
-      <c r="M15" t="n">
-        <v>487</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1261</v>
-      </c>
-      <c r="O15" t="n">
-        <v>34.95</v>
-      </c>
-      <c r="P15" t="n">
-        <v>183</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>816</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="S15" t="n">
-        <v>597</v>
-      </c>
-      <c r="T15" t="n">
-        <v>12224</v>
+        <v>176.709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>